<commit_message>
Konzept v0.4: Lernbegleitung über das Schuljahr und mehrsprachige Nachhilfe
Kernprodukt als Nachhilfe auf zwei Ebenen beschrieben: die geführte
Stunde (täglich) und die Lernbegleitung über das Schuljahr mit
Einstiegs-Check, Stundenplan, Testterminen, Wochenplan,
Wissens-Checks, Schließen alter Lücken und übergeordneter Förderung.
Abgrenzung zu Universal-KI und Lern-App als Tabelle.

Neues Kapitel 2.10 zur Vermittlung des Schulstoffs in der
Herkunftssprache als Brücke zum Deutschen, mit Machbarkeit, Kosten,
Vertriebsweg über Kommunen und Risiken. Produkt-Check im Testbogen
um Stundenplan, Testtermine, Lernstand, Wiederholungsabfragen und
Sprachen ergänzt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0115P4q6mUPpEjGxSG5SLynh
</commit_message>
<xml_diff>
--- a/docs/praxistest/testbogen-ki-tutoren.xlsx
+++ b/docs/praxistest/testbogen-ki-tutoren.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1843" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1850" uniqueCount="327">
   <si>
     <t xml:space="preserve">Praxistest KI-Tutoren – Testbogen</t>
   </si>
@@ -926,9 +926,24 @@
     <t xml:space="preserve">Bundesland, Schulform und Klasse wählbar</t>
   </si>
   <si>
+    <t xml:space="preserve">Stundenplan eintragbar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tests und Klassenarbeiten eintragbar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lernstand wird erhoben (z. B. Einstiegstest)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lernplan bis zur Klassenarbeit</t>
   </si>
   <si>
+    <t xml:space="preserve">Fragt später erneut ab, ob das Wissen sitzt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wiederholung nach Tagen</t>
+  </si>
+  <si>
     <t xml:space="preserve">Probearbeit oder Probeklausur</t>
   </si>
   <si>
@@ -939,6 +954,12 @@
   </si>
   <si>
     <t xml:space="preserve">Belohnungen oder Spielelemente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erklärungen in anderen Sprachen als Deutsch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">welche Sprachen? Qualität?</t>
   </si>
   <si>
     <t xml:space="preserve">Kosten</t>
@@ -16249,7 +16270,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -16685,90 +16706,169 @@
       <c r="H28" s="12"/>
       <c r="I28" s="12"/>
       <c r="J28" s="12"/>
-      <c r="K28" s="28"/>
+      <c r="K28" s="28" t="s">
+        <v>292</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="27" t="s">
-        <v>292</v>
-      </c>
+      <c r="A29" s="4"/>
       <c r="B29" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="28" t="s">
-        <v>294</v>
-      </c>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="28"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4"/>
       <c r="B30" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="28"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4"/>
+      <c r="B31" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="28" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="27" t="s">
-        <v>297</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>298</v>
-      </c>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="10"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
       <c r="K31" s="28"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4"/>
       <c r="B32" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
-      <c r="I32" s="10"/>
-      <c r="J32" s="10"/>
+        <v>296</v>
+      </c>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
       <c r="K32" s="28"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4"/>
       <c r="B33" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="28" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="27" t="s">
+        <v>299</v>
+      </c>
+      <c r="B34" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="12"/>
-      <c r="I33" s="12"/>
-      <c r="J33" s="12"/>
-      <c r="K33" s="28"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="28" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4"/>
+      <c r="B35" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
+      <c r="K35" s="28" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="28"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4"/>
+      <c r="B37" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="28"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4"/>
+      <c r="B38" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="12"/>
+      <c r="J38" s="12"/>
+      <c r="K38" s="28"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C6:J6">
@@ -17024,7 +17124,7 @@
       <formula>"teilweise"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C33:J33">
+  <conditionalFormatting sqref="C29:J29">
     <cfRule type="cellIs" priority="71" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"ja"</formula>
     </cfRule>
@@ -17035,8 +17135,52 @@
       <formula>"teilweise"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C30:J30">
+    <cfRule type="cellIs" priority="74" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+      <formula>"ja"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="75" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>"nein"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="76" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>"teilweise"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C31:J31">
+    <cfRule type="cellIs" priority="77" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+      <formula>"ja"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="78" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>"nein"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="79" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>"teilweise"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C32:J32">
+    <cfRule type="cellIs" priority="80" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+      <formula>"ja"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="81" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>"nein"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="82" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>"teilweise"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C38:J38">
+    <cfRule type="cellIs" priority="83" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+      <formula>"ja"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="84" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>"nein"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="85" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>"teilweise"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6:J28 C33:J33" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6:J32 C38:J38" type="list">
       <formula1>"ja,teilweise,nein,unklar"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -17073,17 +17217,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17091,40 +17235,40 @@
         <v>237</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="M5" s="8" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="N5" s="8" t="s">
         <v>69</v>
@@ -17625,12 +17769,12 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17796,7 +17940,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18256,7 +18400,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>